<commit_message>
Use noncausal encoding semantics for embedding and reranking models
</commit_message>
<xml_diff>
--- a/dist/downloads/model-documents/openbmb-toolbench_ir_bert_based_uncased.xlsx
+++ b/dist/downloads/model-documents/openbmb-toolbench_ir_bert_based_uncased.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="算子表" sheetId="1" r:id="Rab914535cf974ddb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型参数" sheetId="2" r:id="R8be3abfb1f434938"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="算子表" sheetId="1" r:id="R11487e80d4b4434a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型参数" sheetId="2" r:id="R6daff5a7e9494ed2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -627,7 +627,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H2" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I2" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -690,7 +690,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC2" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD2" s="12" t="str">
         <x:v>归一化类型/先后顺序待实现核验</x:v>
@@ -719,7 +719,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H3" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I3" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -782,7 +782,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC3" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD3" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -811,7 +811,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H4" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I4" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -874,7 +874,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC4" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD4" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -903,7 +903,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H5" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I5" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -966,7 +966,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC5" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD5" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -995,7 +995,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H6" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I6" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1058,10 +1058,10 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC6" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD6" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；位置编码与物理layout需实现核验</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；位置编码与物理layout需实现核验</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" hidden="0" customHeight="1">
@@ -1087,7 +1087,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H7" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I7" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1150,7 +1150,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC7" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
       </x:c>
       <x:c r="AD7" s="12" t="str">
         <x:v>softmax(QK^T / sqrt(head_dim) + mask)V（数学参考）</x:v>
@@ -1179,7 +1179,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H8" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I8" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1242,7 +1242,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC8" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD8" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -1271,7 +1271,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H9" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I9" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1334,7 +1334,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC9" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD9" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -1363,7 +1363,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H10" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I10" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1426,7 +1426,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC10" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD10" s="12" t="str">
         <x:v>类型与位置待源码核验</x:v>
@@ -1455,7 +1455,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H11" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I11" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1518,7 +1518,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC11" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD11" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -1547,7 +1547,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H12" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I12" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1610,7 +1610,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC12" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
       </x:c>
       <x:c r="AD12" s="12" t="str">
         <x:v>config.hidden_act=gelu</x:v>
@@ -1639,7 +1639,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H13" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I13" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1702,7 +1702,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC13" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD13" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -1731,7 +1731,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H14" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I14" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1794,7 +1794,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC14" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD14" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -1823,7 +1823,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H15" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I15" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1886,7 +1886,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC15" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD15" s="12" t="str">
         <x:v>归一化类型/先后顺序待实现核验</x:v>
@@ -1915,7 +1915,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H16" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I16" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1978,7 +1978,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC16" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD16" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -2007,7 +2007,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H17" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I17" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2070,7 +2070,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC17" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD17" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -2099,7 +2099,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H18" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I18" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2162,7 +2162,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC18" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD18" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -2191,7 +2191,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H19" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I19" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2254,10 +2254,10 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC19" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD19" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；位置编码与物理layout需实现核验</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；位置编码与物理layout需实现核验</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="24" hidden="0" customHeight="1">
@@ -2283,7 +2283,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H20" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I20" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2346,7 +2346,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC20" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
       </x:c>
       <x:c r="AD20" s="12" t="str">
         <x:v>softmax(QK^T / sqrt(head_dim) + mask)V（数学参考）</x:v>
@@ -2375,7 +2375,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H21" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I21" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2438,7 +2438,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC21" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD21" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -2467,7 +2467,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H22" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I22" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2530,7 +2530,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC22" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD22" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -2559,7 +2559,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H23" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I23" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2622,7 +2622,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC23" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD23" s="12" t="str">
         <x:v>类型与位置待源码核验</x:v>
@@ -2651,7 +2651,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H24" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I24" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2714,7 +2714,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC24" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD24" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -2743,7 +2743,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H25" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I25" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2806,7 +2806,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC25" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
       </x:c>
       <x:c r="AD25" s="12" t="str">
         <x:v>config.hidden_act=gelu</x:v>
@@ -2835,7 +2835,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H26" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I26" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2898,7 +2898,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC26" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD26" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -2927,7 +2927,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H27" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I27" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2990,7 +2990,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC27" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD27" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -3019,7 +3019,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H28" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I28" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3082,7 +3082,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC28" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD28" s="12" t="str">
         <x:v>归一化类型/先后顺序待实现核验</x:v>
@@ -3111,7 +3111,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H29" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I29" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3174,7 +3174,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC29" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD29" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -3203,7 +3203,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H30" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I30" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3266,7 +3266,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC30" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD30" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -3295,7 +3295,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H31" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I31" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3358,7 +3358,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC31" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD31" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -3387,7 +3387,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H32" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I32" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3450,10 +3450,10 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC32" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD32" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；位置编码与物理layout需实现核验</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；位置编码与物理layout需实现核验</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="24" hidden="0" customHeight="1">
@@ -3479,7 +3479,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H33" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I33" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3542,7 +3542,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC33" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
       </x:c>
       <x:c r="AD33" s="12" t="str">
         <x:v>softmax(QK^T / sqrt(head_dim) + mask)V（数学参考）</x:v>
@@ -3571,7 +3571,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H34" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I34" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3634,7 +3634,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC34" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD34" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -3663,7 +3663,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H35" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I35" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3726,7 +3726,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC35" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD35" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -3755,7 +3755,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H36" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I36" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3818,7 +3818,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC36" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD36" s="12" t="str">
         <x:v>类型与位置待源码核验</x:v>
@@ -3847,7 +3847,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H37" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I37" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3910,7 +3910,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC37" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD37" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -3939,7 +3939,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H38" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I38" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4002,7 +4002,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC38" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
       </x:c>
       <x:c r="AD38" s="12" t="str">
         <x:v>config.hidden_act=gelu</x:v>
@@ -4031,7 +4031,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H39" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I39" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4094,7 +4094,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC39" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD39" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -4123,7 +4123,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H40" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I40" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4186,7 +4186,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC40" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD40" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -4215,7 +4215,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H41" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I41" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4278,7 +4278,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC41" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD41" s="12" t="str">
         <x:v>归一化类型/先后顺序待实现核验</x:v>
@@ -4307,7 +4307,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H42" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I42" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4370,7 +4370,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC42" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD42" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -4399,7 +4399,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H43" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I43" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4462,7 +4462,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC43" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD43" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -4491,7 +4491,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H44" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I44" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4554,7 +4554,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC44" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD44" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -4583,7 +4583,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H45" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I45" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4646,10 +4646,10 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC45" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD45" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；位置编码与物理layout需实现核验</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；位置编码与物理layout需实现核验</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="24" hidden="0" customHeight="1">
@@ -4675,7 +4675,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H46" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I46" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4738,7 +4738,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC46" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
       </x:c>
       <x:c r="AD46" s="12" t="str">
         <x:v>softmax(QK^T / sqrt(head_dim) + mask)V（数学参考）</x:v>
@@ -4767,7 +4767,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H47" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I47" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4830,7 +4830,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC47" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD47" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -4859,7 +4859,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H48" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I48" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4922,7 +4922,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC48" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD48" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -4951,7 +4951,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H49" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I49" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5014,7 +5014,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC49" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD49" s="12" t="str">
         <x:v>类型与位置待源码核验</x:v>
@@ -5043,7 +5043,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H50" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I50" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5106,7 +5106,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC50" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD50" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -5135,7 +5135,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H51" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I51" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5198,7 +5198,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC51" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
       </x:c>
       <x:c r="AD51" s="12" t="str">
         <x:v>config.hidden_act=gelu</x:v>
@@ -5227,7 +5227,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H52" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I52" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5290,7 +5290,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC52" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD52" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -5319,7 +5319,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H53" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I53" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5382,7 +5382,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC53" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD53" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -5411,7 +5411,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H54" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I54" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5474,7 +5474,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC54" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD54" s="12" t="str">
         <x:v>归一化类型/先后顺序待实现核验</x:v>
@@ -5503,7 +5503,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H55" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I55" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5566,7 +5566,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC55" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD55" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -5595,7 +5595,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H56" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I56" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5658,7 +5658,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC56" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD56" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -5687,7 +5687,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H57" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I57" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5750,7 +5750,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC57" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD57" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -5779,7 +5779,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H58" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I58" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5842,10 +5842,10 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC58" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD58" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；位置编码与物理layout需实现核验</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；位置编码与物理layout需实现核验</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="24" hidden="0" customHeight="1">
@@ -5871,7 +5871,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H59" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I59" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5934,7 +5934,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC59" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
       </x:c>
       <x:c r="AD59" s="12" t="str">
         <x:v>softmax(QK^T / sqrt(head_dim) + mask)V（数学参考）</x:v>
@@ -5963,7 +5963,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H60" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I60" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6026,7 +6026,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC60" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD60" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -6055,7 +6055,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H61" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I61" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6118,7 +6118,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC61" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD61" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -6147,7 +6147,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H62" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I62" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6210,7 +6210,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC62" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD62" s="12" t="str">
         <x:v>类型与位置待源码核验</x:v>
@@ -6239,7 +6239,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H63" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I63" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6302,7 +6302,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC63" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD63" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -6331,7 +6331,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H64" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I64" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6394,7 +6394,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC64" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
       </x:c>
       <x:c r="AD64" s="12" t="str">
         <x:v>config.hidden_act=gelu</x:v>
@@ -6423,7 +6423,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H65" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I65" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6486,7 +6486,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC65" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD65" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -6515,7 +6515,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H66" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I66" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6578,7 +6578,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC66" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD66" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -6607,7 +6607,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H67" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I67" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6670,7 +6670,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC67" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD67" s="12" t="str">
         <x:v>归一化类型/先后顺序待实现核验</x:v>
@@ -6699,7 +6699,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H68" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I68" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6762,7 +6762,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC68" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD68" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -6791,7 +6791,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H69" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I69" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6854,7 +6854,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC69" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD69" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -6883,7 +6883,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H70" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I70" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6946,7 +6946,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC70" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD70" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -6975,7 +6975,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H71" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I71" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7038,10 +7038,10 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC71" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD71" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；位置编码与物理layout需实现核验</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；位置编码与物理layout需实现核验</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="24" hidden="0" customHeight="1">
@@ -7067,7 +7067,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H72" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I72" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7130,7 +7130,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC72" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
       </x:c>
       <x:c r="AD72" s="12" t="str">
         <x:v>softmax(QK^T / sqrt(head_dim) + mask)V（数学参考）</x:v>
@@ -7159,7 +7159,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H73" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I73" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7222,7 +7222,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC73" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD73" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -7251,7 +7251,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H74" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I74" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7314,7 +7314,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC74" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD74" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -7343,7 +7343,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H75" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I75" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7406,7 +7406,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC75" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD75" s="12" t="str">
         <x:v>类型与位置待源码核验</x:v>
@@ -7435,7 +7435,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H76" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I76" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7498,7 +7498,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC76" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD76" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -7527,7 +7527,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H77" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I77" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7590,7 +7590,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC77" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
       </x:c>
       <x:c r="AD77" s="12" t="str">
         <x:v>config.hidden_act=gelu</x:v>
@@ -7619,7 +7619,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H78" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I78" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7682,7 +7682,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC78" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD78" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -7711,7 +7711,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H79" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I79" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7774,7 +7774,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC79" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD79" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -7803,7 +7803,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H80" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I80" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7866,7 +7866,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC80" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD80" s="12" t="str">
         <x:v>归一化类型/先后顺序待实现核验</x:v>
@@ -7895,7 +7895,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H81" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I81" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7958,7 +7958,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC81" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD81" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -7987,7 +7987,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H82" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I82" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8050,7 +8050,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC82" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD82" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -8079,7 +8079,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H83" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I83" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8142,7 +8142,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC83" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD83" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -8171,7 +8171,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H84" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I84" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8234,10 +8234,10 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC84" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD84" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；位置编码与物理layout需实现核验</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；位置编码与物理layout需实现核验</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="24" hidden="0" customHeight="1">
@@ -8263,7 +8263,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H85" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I85" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8326,7 +8326,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC85" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
       </x:c>
       <x:c r="AD85" s="12" t="str">
         <x:v>softmax(QK^T / sqrt(head_dim) + mask)V（数学参考）</x:v>
@@ -8355,7 +8355,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H86" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I86" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8418,7 +8418,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC86" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD86" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -8447,7 +8447,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H87" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I87" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8510,7 +8510,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC87" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD87" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -8539,7 +8539,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H88" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I88" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8602,7 +8602,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC88" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD88" s="12" t="str">
         <x:v>类型与位置待源码核验</x:v>
@@ -8631,7 +8631,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H89" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I89" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8694,7 +8694,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC89" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD89" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -8723,7 +8723,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H90" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I90" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8786,7 +8786,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC90" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
       </x:c>
       <x:c r="AD90" s="12" t="str">
         <x:v>config.hidden_act=gelu</x:v>
@@ -8815,7 +8815,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H91" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I91" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8878,7 +8878,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC91" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD91" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -8907,7 +8907,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H92" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I92" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8970,7 +8970,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC92" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD92" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -8999,7 +8999,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H93" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I93" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9062,7 +9062,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC93" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD93" s="12" t="str">
         <x:v>归一化类型/先后顺序待实现核验</x:v>
@@ -9091,7 +9091,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H94" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I94" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9154,7 +9154,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC94" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD94" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -9183,7 +9183,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H95" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I95" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9246,7 +9246,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC95" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD95" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -9275,7 +9275,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H96" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I96" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9338,7 +9338,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC96" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD96" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -9367,7 +9367,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H97" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I97" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9430,10 +9430,10 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC97" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD97" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；位置编码与物理layout需实现核验</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；位置编码与物理layout需实现核验</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="24" hidden="0" customHeight="1">
@@ -9459,7 +9459,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H98" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I98" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9522,7 +9522,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC98" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
       </x:c>
       <x:c r="AD98" s="12" t="str">
         <x:v>softmax(QK^T / sqrt(head_dim) + mask)V（数学参考）</x:v>
@@ -9551,7 +9551,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H99" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I99" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9614,7 +9614,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC99" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD99" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -9643,7 +9643,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H100" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I100" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9706,7 +9706,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC100" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD100" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -9735,7 +9735,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H101" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I101" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9798,7 +9798,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC101" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD101" s="12" t="str">
         <x:v>类型与位置待源码核验</x:v>
@@ -9827,7 +9827,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H102" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I102" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9890,7 +9890,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC102" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD102" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -9919,7 +9919,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H103" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I103" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9982,7 +9982,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC103" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
       </x:c>
       <x:c r="AD103" s="12" t="str">
         <x:v>config.hidden_act=gelu</x:v>
@@ -10011,7 +10011,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H104" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I104" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10074,7 +10074,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC104" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD104" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -10103,7 +10103,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H105" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I105" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10166,7 +10166,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC105" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD105" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -10195,7 +10195,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H106" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I106" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10258,7 +10258,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC106" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD106" s="12" t="str">
         <x:v>归一化类型/先后顺序待实现核验</x:v>
@@ -10287,7 +10287,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H107" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I107" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10350,7 +10350,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC107" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD107" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -10379,7 +10379,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H108" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I108" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10442,7 +10442,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC108" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD108" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -10471,7 +10471,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H109" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I109" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10534,7 +10534,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC109" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD109" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -10563,7 +10563,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H110" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I110" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10626,10 +10626,10 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC110" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD110" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；位置编码与物理layout需实现核验</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；位置编码与物理layout需实现核验</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="24" hidden="0" customHeight="1">
@@ -10655,7 +10655,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H111" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I111" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10718,7 +10718,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC111" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
       </x:c>
       <x:c r="AD111" s="12" t="str">
         <x:v>softmax(QK^T / sqrt(head_dim) + mask)V（数学参考）</x:v>
@@ -10747,7 +10747,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H112" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I112" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10810,7 +10810,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC112" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD112" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -10839,7 +10839,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H113" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I113" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10902,7 +10902,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC113" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD113" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -10931,7 +10931,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H114" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I114" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10994,7 +10994,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC114" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD114" s="12" t="str">
         <x:v>类型与位置待源码核验</x:v>
@@ -11023,7 +11023,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H115" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I115" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11086,7 +11086,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC115" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD115" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -11115,7 +11115,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H116" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I116" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11178,7 +11178,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC116" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
       </x:c>
       <x:c r="AD116" s="12" t="str">
         <x:v>config.hidden_act=gelu</x:v>
@@ -11207,7 +11207,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H117" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I117" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11270,7 +11270,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC117" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD117" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -11299,7 +11299,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H118" s="11" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I118" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11362,7 +11362,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC118" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD118" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -11391,7 +11391,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H119" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I119" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11454,7 +11454,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC119" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD119" s="12" t="str">
         <x:v>归一化类型/先后顺序待实现核验</x:v>
@@ -11483,7 +11483,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H120" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I120" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11546,7 +11546,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC120" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD120" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -11575,7 +11575,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H121" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I121" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11638,7 +11638,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC121" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD121" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -11667,7 +11667,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H122" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I122" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11730,7 +11730,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC122" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD122" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -11759,7 +11759,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H123" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I123" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11822,10 +11822,10 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC123" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD123" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；位置编码与物理layout需实现核验</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；位置编码与物理layout需实现核验</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="24" hidden="0" customHeight="1">
@@ -11851,7 +11851,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H124" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I124" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11914,7 +11914,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC124" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
       </x:c>
       <x:c r="AD124" s="12" t="str">
         <x:v>softmax(QK^T / sqrt(head_dim) + mask)V（数学参考）</x:v>
@@ -11943,7 +11943,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H125" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I125" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12006,7 +12006,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC125" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD125" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -12035,7 +12035,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H126" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I126" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12098,7 +12098,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC126" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD126" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -12127,7 +12127,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H127" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I127" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12190,7 +12190,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC127" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD127" s="12" t="str">
         <x:v>类型与位置待源码核验</x:v>
@@ -12219,7 +12219,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H128" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I128" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12282,7 +12282,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC128" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD128" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -12311,7 +12311,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H129" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I129" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12374,7 +12374,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC129" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
       </x:c>
       <x:c r="AD129" s="12" t="str">
         <x:v>config.hidden_act=gelu</x:v>
@@ -12403,7 +12403,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H130" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I130" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12466,7 +12466,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC130" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD130" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -12495,7 +12495,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H131" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I131" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12558,7 +12558,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC131" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD131" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -12587,7 +12587,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H132" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I132" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12650,7 +12650,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC132" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD132" s="12" t="str">
         <x:v>归一化类型/先后顺序待实现核验</x:v>
@@ -12679,7 +12679,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H133" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I133" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12742,7 +12742,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC133" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD133" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -12771,7 +12771,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H134" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I134" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12834,7 +12834,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC134" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD134" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -12863,7 +12863,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H135" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I135" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12926,7 +12926,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC135" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD135" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -12955,7 +12955,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H136" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I136" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13018,10 +13018,10 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC136" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD136" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；位置编码与物理layout需实现核验</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；位置编码与物理layout需实现核验</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="24" hidden="0" customHeight="1">
@@ -13047,7 +13047,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H137" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I137" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13110,7 +13110,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC137" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
       </x:c>
       <x:c r="AD137" s="12" t="str">
         <x:v>softmax(QK^T / sqrt(head_dim) + mask)V（数学参考）</x:v>
@@ -13139,7 +13139,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H138" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I138" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13202,7 +13202,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC138" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD138" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -13231,7 +13231,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H139" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I139" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13294,7 +13294,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC139" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD139" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -13323,7 +13323,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H140" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I140" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13386,7 +13386,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC140" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD140" s="12" t="str">
         <x:v>类型与位置待源码核验</x:v>
@@ -13415,7 +13415,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H141" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I141" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13478,7 +13478,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC141" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD141" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -13507,7 +13507,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H142" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I142" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13570,7 +13570,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC142" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
       </x:c>
       <x:c r="AD142" s="12" t="str">
         <x:v>config.hidden_act=gelu</x:v>
@@ -13599,7 +13599,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H143" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I143" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13662,7 +13662,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC143" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD143" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -13691,7 +13691,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H144" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I144" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13754,7 +13754,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC144" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD144" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -13783,7 +13783,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H145" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I145" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13846,7 +13846,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC145" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD145" s="12" t="str">
         <x:v>归一化类型/先后顺序待实现核验</x:v>
@@ -13875,7 +13875,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H146" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I146" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13938,7 +13938,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC146" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD146" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -13967,7 +13967,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H147" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I147" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14030,7 +14030,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC147" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD147" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -14059,7 +14059,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H148" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I148" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14122,7 +14122,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC148" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；独立逻辑矩阵，不断言实际融合与存储</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；独立逻辑矩阵，不断言实际融合与存储</x:v>
       </x:c>
       <x:c r="AD148" s="12" t="str">
         <x:v>Y=X@W^T; width=heads*head_dim</x:v>
@@ -14151,7 +14151,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H149" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I149" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14214,10 +14214,10 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC149" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD149" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；位置编码与物理layout需实现核验</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；位置编码与物理layout需实现核验</x:v>
       </x:c>
     </x:row>
     <x:row r="150" ht="24" hidden="0" customHeight="1">
@@ -14243,7 +14243,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H150" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I150" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14306,7 +14306,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC150" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；稀疏选块/线性分支需按实现，不能据此声称稠密执行或峰值中间内存</x:v>
       </x:c>
       <x:c r="AD150" s="12" t="str">
         <x:v>softmax(QK^T / sqrt(head_dim) + mask)V（数学参考）</x:v>
@@ -14335,7 +14335,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H151" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I151" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14398,7 +14398,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC151" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD151" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -14427,7 +14427,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H152" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I152" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14490,7 +14490,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC152" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD152" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -14519,7 +14519,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H153" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I153" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14582,7 +14582,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC153" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD153" s="12" t="str">
         <x:v>类型与位置待源码核验</x:v>
@@ -14611,7 +14611,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H154" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I154" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14674,7 +14674,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC154" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD154" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -14703,7 +14703,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H155" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I155" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14766,7 +14766,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC155" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；是否额外gate矩阵与门控分支维度需要实现；不能仅由silu推定完整SwiGLU</x:v>
       </x:c>
       <x:c r="AD155" s="12" t="str">
         <x:v>config.hidden_act=gelu</x:v>
@@ -14795,7 +14795,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H156" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I156" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14858,7 +14858,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC156" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD156" s="12" t="str">
         <x:v>Y=X@W^T</x:v>
@@ -14887,7 +14887,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H157" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I157" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14950,7 +14950,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC157" s="12" t="str">
-        <x:v>文本编码/检索；Q/K/V同输入长度L_text，无解码历史KV缓存；S_verify不适用；</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；</x:v>
       </x:c>
       <x:c r="AD157" s="12" t="str">
         <x:v>Y=X+branch（参考，实际残差策略未核验）</x:v>
@@ -14979,7 +14979,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H158" s="12" t="str">
-        <x:v>L_text由输入决定；verify长度和历史KV不适用</x:v>
+        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I158" s="12" t="str">
         <x:v>未核验</x:v>
@@ -15042,7 +15042,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="AC158" s="12" t="str">
-        <x:v>文本编码/检索；L_text为输入长度，无解码历史KV缓存；embedding、lm_head、模态连接器、压缩器、AudioVAE、扩散/动作/检索头需独立源码；不因主干展开而声称全图已完成</x:v>
+        <x:v>文本编码/检索；Q/K/V同输入长度L_text；S_verify不适用；BERT非decoder，无历史KV缓存；embedding、lm_head、模态连接器、压缩器、AudioVAE、扩散/动作/检索头需独立源码；不因主干展开而声称全图已完成</x:v>
       </x:c>
       <x:c r="AD158" s="12" t="str">
         <x:v>未核验</x:v>
@@ -15145,7 +15145,7 @@
         <x:v>https://huggingface.co/ToolBench/ToolBench_IR_bert_based_uncased/resolve/cf4a904c33cde549643aa6d9091146e68ed4932f/config.json</x:v>
       </x:c>
       <x:c r="E4" s="28" t="str">
-        <x:v>BERT编码器无verify阶段</x:v>
+        <x:v>编码/检索视图不套用verify阶段</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="24" hidden="0" customHeight="1">
@@ -15506,7 +15506,7 @@
         <x:v>阶段</x:v>
       </x:c>
       <x:c r="B23" s="28" t="str">
-        <x:v>文本编码/检索，无解码历史KV缓存</x:v>
+        <x:v>单次文本编码/检索；Q/K/V同L_text；历史缓存路径不在本逻辑视图内</x:v>
       </x:c>
       <x:c r="C23" s="28"/>
       <x:c r="D23" s="28"/>

</xml_diff>

<commit_message>
Document retrieval input stages with pinned implementation sources
</commit_message>
<xml_diff>
--- a/dist/downloads/model-documents/openbmb-toolbench_ir_bert_based_uncased.xlsx
+++ b/dist/downloads/model-documents/openbmb-toolbench_ir_bert_based_uncased.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="算子表" sheetId="1" r:id="R11487e80d4b4434a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型参数" sheetId="2" r:id="R6daff5a7e9494ed2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="算子表" sheetId="1" r:id="R8b89918f69ee4ce8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型参数" sheetId="2" r:id="Ra480120fbef54fd5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -627,7 +627,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H2" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I2" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -719,7 +719,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H3" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I3" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -811,7 +811,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H4" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I4" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -903,7 +903,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H5" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I5" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -995,7 +995,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H6" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I6" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1087,7 +1087,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H7" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I7" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1179,7 +1179,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H8" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I8" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1271,7 +1271,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H9" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I9" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1363,7 +1363,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H10" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I10" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1455,7 +1455,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H11" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I11" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1547,7 +1547,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H12" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I12" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1639,7 +1639,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H13" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I13" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1731,7 +1731,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H14" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I14" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1823,7 +1823,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H15" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I15" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -1915,7 +1915,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H16" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I16" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2007,7 +2007,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H17" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I17" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2099,7 +2099,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H18" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I18" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2191,7 +2191,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H19" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I19" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2283,7 +2283,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H20" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I20" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2375,7 +2375,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H21" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I21" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2467,7 +2467,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H22" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I22" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2559,7 +2559,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H23" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I23" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2651,7 +2651,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H24" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I24" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2743,7 +2743,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H25" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I25" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2835,7 +2835,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H26" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I26" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -2927,7 +2927,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H27" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I27" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3019,7 +3019,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H28" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I28" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3111,7 +3111,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H29" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I29" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3203,7 +3203,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H30" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I30" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3295,7 +3295,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H31" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I31" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3387,7 +3387,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H32" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I32" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3479,7 +3479,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H33" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I33" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3571,7 +3571,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H34" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I34" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3663,7 +3663,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H35" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I35" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3755,7 +3755,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H36" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I36" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3847,7 +3847,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H37" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I37" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -3939,7 +3939,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H38" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I38" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4031,7 +4031,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H39" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I39" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4123,7 +4123,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H40" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I40" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4215,7 +4215,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H41" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I41" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4307,7 +4307,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H42" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I42" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4399,7 +4399,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H43" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I43" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4491,7 +4491,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H44" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I44" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4583,7 +4583,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H45" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I45" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4675,7 +4675,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H46" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I46" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4767,7 +4767,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H47" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I47" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4859,7 +4859,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H48" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I48" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -4951,7 +4951,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H49" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I49" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5043,7 +5043,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H50" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I50" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5135,7 +5135,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H51" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I51" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5227,7 +5227,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H52" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I52" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5319,7 +5319,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H53" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I53" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5411,7 +5411,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H54" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I54" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5503,7 +5503,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H55" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I55" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5595,7 +5595,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H56" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I56" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5687,7 +5687,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H57" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I57" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5779,7 +5779,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H58" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I58" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5871,7 +5871,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H59" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I59" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -5963,7 +5963,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H60" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I60" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6055,7 +6055,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H61" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I61" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6147,7 +6147,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H62" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I62" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6239,7 +6239,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H63" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I63" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6331,7 +6331,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H64" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I64" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6423,7 +6423,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H65" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I65" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6515,7 +6515,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H66" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I66" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6607,7 +6607,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H67" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I67" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6699,7 +6699,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H68" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I68" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6791,7 +6791,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H69" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I69" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6883,7 +6883,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H70" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I70" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -6975,7 +6975,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H71" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I71" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7067,7 +7067,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H72" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I72" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7159,7 +7159,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H73" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I73" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7251,7 +7251,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H74" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I74" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7343,7 +7343,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H75" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I75" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7435,7 +7435,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H76" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I76" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7527,7 +7527,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H77" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I77" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7619,7 +7619,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H78" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I78" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7711,7 +7711,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H79" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I79" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7803,7 +7803,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H80" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I80" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7895,7 +7895,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H81" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I81" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -7987,7 +7987,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H82" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I82" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8079,7 +8079,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H83" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I83" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8171,7 +8171,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H84" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I84" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8263,7 +8263,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H85" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I85" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8355,7 +8355,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H86" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I86" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8447,7 +8447,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H87" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I87" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8539,7 +8539,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H88" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I88" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8631,7 +8631,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H89" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I89" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8723,7 +8723,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H90" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I90" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8815,7 +8815,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H91" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I91" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8907,7 +8907,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H92" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I92" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -8999,7 +8999,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H93" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I93" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9091,7 +9091,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H94" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I94" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9183,7 +9183,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H95" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I95" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9275,7 +9275,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H96" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I96" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9367,7 +9367,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H97" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I97" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9459,7 +9459,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H98" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I98" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9551,7 +9551,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H99" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I99" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9643,7 +9643,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H100" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I100" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9735,7 +9735,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H101" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I101" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9827,7 +9827,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H102" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I102" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -9919,7 +9919,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H103" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I103" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10011,7 +10011,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H104" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I104" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10103,7 +10103,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H105" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I105" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10195,7 +10195,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H106" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I106" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10287,7 +10287,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H107" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I107" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10379,7 +10379,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H108" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I108" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10471,7 +10471,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H109" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I109" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10563,7 +10563,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H110" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I110" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10655,7 +10655,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H111" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I111" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10747,7 +10747,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H112" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I112" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10839,7 +10839,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H113" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I113" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -10931,7 +10931,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H114" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I114" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11023,7 +11023,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H115" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I115" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11115,7 +11115,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H116" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I116" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11207,7 +11207,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H117" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I117" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11299,7 +11299,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H118" s="11" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I118" s="11" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11391,7 +11391,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H119" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I119" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11483,7 +11483,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H120" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I120" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11575,7 +11575,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H121" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I121" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11667,7 +11667,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H122" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I122" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11759,7 +11759,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H123" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I123" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11851,7 +11851,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H124" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I124" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -11943,7 +11943,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H125" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I125" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12035,7 +12035,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H126" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I126" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12127,7 +12127,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H127" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I127" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12219,7 +12219,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H128" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I128" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12311,7 +12311,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H129" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I129" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12403,7 +12403,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H130" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I130" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12495,7 +12495,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H131" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I131" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12587,7 +12587,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H132" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I132" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12679,7 +12679,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H133" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I133" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12771,7 +12771,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H134" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I134" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12863,7 +12863,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H135" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I135" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -12955,7 +12955,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H136" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I136" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13047,7 +13047,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H137" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I137" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13139,7 +13139,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H138" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I138" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13231,7 +13231,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H139" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I139" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13323,7 +13323,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H140" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I140" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13415,7 +13415,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H141" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I141" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13507,7 +13507,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H142" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I142" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13599,7 +13599,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H143" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I143" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13691,7 +13691,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H144" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I144" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13783,7 +13783,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H145" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I145" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13875,7 +13875,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H146" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I146" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -13967,7 +13967,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H147" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I147" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14059,7 +14059,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H148" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I148" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14151,7 +14151,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H149" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I149" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14243,7 +14243,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H150" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I150" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14335,7 +14335,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H151" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I151" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14427,7 +14427,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H152" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I152" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14519,7 +14519,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H153" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I153" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14611,7 +14611,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H154" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I154" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14703,7 +14703,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H155" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I155" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14795,7 +14795,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H156" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I156" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14887,7 +14887,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H157" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I157" s="12" t="str">
         <x:v>config=float32；激活/累加类型未核验</x:v>
@@ -14979,7 +14979,7 @@
         <x:v>B,L_text；编码输入长度</x:v>
       </x:c>
       <x:c r="H158" s="12" t="str">
-        <x:v>L_text由输入决定；单次非因果编码，不套verify历史KV假设</x:v>
+        <x:v>L_text由输入决定；单次编码/检索，不套verify历史KV假设</x:v>
       </x:c>
       <x:c r="I158" s="12" t="str">
         <x:v>未核验</x:v>
@@ -15506,7 +15506,7 @@
         <x:v>阶段</x:v>
       </x:c>
       <x:c r="B23" s="28" t="str">
-        <x:v>单次文本编码/检索；Q/K/V同L_text；历史缓存路径不在本逻辑视图内</x:v>
+        <x:v>单次编码/检索；Q/K/V同L_text；历史缓存路径不在本逻辑视图内</x:v>
       </x:c>
       <x:c r="C23" s="28"/>
       <x:c r="D23" s="28"/>
@@ -15550,7 +15550,7 @@
         <x:v>S语义</x:v>
       </x:c>
       <x:c r="B27" s="28" t="str">
-        <x:v>模板S保留定义，本编码器不适用；使用L_text</x:v>
+        <x:v>模板S保留定义，本任务阶段不适用；使用L_text</x:v>
       </x:c>
       <x:c r="C27" s="28"/>
       <x:c r="D27" s="28"/>

</xml_diff>